<commit_message>
[0.0.7] - 2025-10-17 Completing PTZ Bench Testing Notes
</commit_message>
<xml_diff>
--- a/PTZ/Device_Inventory.xlsx
+++ b/PTZ/Device_Inventory.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/99d2d0efc5e421e1/Working_Files/CPC_Production/PTZ/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_F25DC773A252ABDACC1048B0395B70645BDE58E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D8B20B47-D487-42C1-8CB0-947E5118EECD}"/>
+  <xr:revisionPtr revIDLastSave="72" documentId="11_F25DC773A252ABDACC1048B0395B70645BDE58E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{85031B00-4417-4305-93D0-3B3AF448A3D1}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,9 +25,107 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
-  <si>
-    <t>Device Inventory</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="31">
+  <si>
+    <t>Device</t>
+  </si>
+  <si>
+    <t>IP</t>
+  </si>
+  <si>
+    <t>Mac</t>
+  </si>
+  <si>
+    <t>User ID</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>Home Router (eero)</t>
+  </si>
+  <si>
+    <t>Connections</t>
+  </si>
+  <si>
+    <t>Switch</t>
+  </si>
+  <si>
+    <t>Controller</t>
+  </si>
+  <si>
+    <t>* Lan Port 1
+     * Port 2 of Home Router (eero)
+* POE Ports
+     *  Port 1 -- Camera 3
+     *  Port 2 -- Camera 4
+     *  Port 8 -- Controller</t>
+  </si>
+  <si>
+    <t>* Ethernet -- Switch Cloud POE Port 1
+* HDMI -- NA</t>
+  </si>
+  <si>
+    <t>*  Port 2 -- Switch</t>
+  </si>
+  <si>
+    <t>* Ethernet -- Switch Cloud POE Port 2
+* HDMI -- NA</t>
+  </si>
+  <si>
+    <t>* Ethernet -- Switch Cloud POE Port 8</t>
+  </si>
+  <si>
+    <t>Model / Brand</t>
+  </si>
+  <si>
+    <t>eero / J9C6-O6M8-54FM-HBO1</t>
+  </si>
+  <si>
+    <t>48:dd:0c:f5:ba:01</t>
+  </si>
+  <si>
+    <t>196.168.4.1</t>
+  </si>
+  <si>
+    <t>GPS208V3</t>
+  </si>
+  <si>
+    <t>ACN Technologies / LV20N</t>
+  </si>
+  <si>
+    <t>Camera 3 (LV20N 3)</t>
+  </si>
+  <si>
+    <t>196.168.4.223 : 5961</t>
+  </si>
+  <si>
+    <t>00:04:05:01:a2:8b</t>
+  </si>
+  <si>
+    <t>Protocol</t>
+  </si>
+  <si>
+    <t>NDI</t>
+  </si>
+  <si>
+    <t>Camera 4 (LV20N 4)</t>
+  </si>
+  <si>
+    <t>196.168.4.225 : 5961</t>
+  </si>
+  <si>
+    <t>00:04:05:15:80:9c</t>
+  </si>
+  <si>
+    <t>XIAMEN SMARTTEC CO. LTD.
+RV 1126 RV 1109</t>
+  </si>
+  <si>
+    <t>196.168.4.224</t>
+  </si>
+  <si>
+    <t>3c:6a:2c:d7:c2:8e</t>
   </si>
 </sst>
 </file>
@@ -63,8 +161,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -80,6 +187,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -345,12 +456,136 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2"/>
+  <dimension ref="B2:G9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="13.7109375" customWidth="1"/>
+    <col min="3" max="3" width="28.5703125" customWidth="1"/>
+    <col min="4" max="4" width="40.7109375" customWidth="1"/>
+    <col min="5" max="7" width="35.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" ht="91.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B5" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B6" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" t="s">
+        <v>24</v>
+      </c>
+      <c r="F7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B8" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B9" s="2" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[0.0.8] - 2025-10-18 Completing PTZ Installed -- Ready for Startup
</commit_message>
<xml_diff>
--- a/PTZ/Device_Inventory.xlsx
+++ b/PTZ/Device_Inventory.xlsx
@@ -8,13 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/99d2d0efc5e421e1/Working_Files/CPC_Production/PTZ/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="72" documentId="11_F25DC773A252ABDACC1048B0395B70645BDE58E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{85031B00-4417-4305-93D0-3B3AF448A3D1}"/>
+  <xr:revisionPtr revIDLastSave="88" documentId="11_F25DC773A252ABDACC1048B0395B70645BDE58E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{77AD831F-C28F-4411-96DD-605DDA05C55B}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bench Setup" sheetId="1" r:id="rId1"/>
+    <sheet name="As Installed" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'As Installed'!$B$2:$G$9</definedName>
+  </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -25,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="36">
   <si>
     <t>Device</t>
   </si>
@@ -126,6 +130,21 @@
   </si>
   <si>
     <t>3c:6a:2c:d7:c2:8e</t>
+  </si>
+  <si>
+    <t>Legacy Switch</t>
+  </si>
+  <si>
+    <t>*  Lan Port 2</t>
+  </si>
+  <si>
+    <t>10.0.1.49 : 5961</t>
+  </si>
+  <si>
+    <t>10.0.1.50 : 5961</t>
+  </si>
+  <si>
+    <t>10.0.1.48</t>
   </si>
 </sst>
 </file>
@@ -149,7 +168,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -157,11 +176,146 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thick">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thick">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top style="thick">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -172,6 +326,35 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -591,4 +774,156 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BAB00A4-BC53-493E-B6DC-080D1237B9FC}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B1:G10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="13.7109375" customWidth="1"/>
+    <col min="3" max="3" width="28.5703125" customWidth="1"/>
+    <col min="4" max="4" width="40.7109375" customWidth="1"/>
+    <col min="5" max="7" width="35.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" ht="91.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="13" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5" s="14" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" s="11"/>
+      <c r="D6" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G6" s="14" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="G7" s="15"/>
+    </row>
+    <row r="8" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="15"/>
+    </row>
+    <row r="9" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="18"/>
+    </row>
+    <row r="10" spans="2:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup scale="64" orientation="landscape" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"-,Bold"&amp;18CPC PTZ Camera Device BOM</oddHeader>
+    <oddFooter>&amp;LPrinted &amp;D at &amp;T</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>